<commit_message>
Updated files and added new docs
Updated files and added new docs
</commit_message>
<xml_diff>
--- a/District_GIS_Parakh_CMMI_L5_Artifacts/District GIS Parakh Artefacts/Katni/DMF Mining releted for DMF alloction before surveys/Baseline Survey Formate.xlsx
+++ b/District_GIS_Parakh_CMMI_L5_Artifacts/District GIS Parakh Artefacts/Katni/DMF Mining releted for DMF alloction before surveys/Baseline Survey Formate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Department_Katni\Mining+DMF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Organization_Docs\District_GIS_Parakh_CMMI_L5_Artifacts\District GIS Parakh Artefacts\Katni\DMF Mining releted for DMF alloction before surveys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27334A17-9CB4-4037-813B-E4E67445DC30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B97C0FEB-A3A7-4B79-9400-10FD820E684D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D861F57-A09B-4C11-9630-4BC99E47DD6F}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{2D861F57-A09B-4C11-9630-4BC99E47DD6F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
     <t>https://forms.gle/SbWju6ABYh6Mc8W86</t>
   </si>
   <si>
-    <t>sanitation</t>
-  </si>
-  <si>
     <t>https://forms.gle/9bFfFLHFsJ9YCAkR9</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>https://forms.gle/q4EpxLX5L334Kxio6</t>
+  </si>
+  <si>
+    <t>sanitation Cleaniiless</t>
   </si>
 </sst>
 </file>
@@ -162,12 +162,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -235,7 +241,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -254,6 +260,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -611,7 +620,7 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -625,7 +634,7 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -639,7 +648,7 @@
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -649,15 +658,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>3</v>
@@ -667,137 +676,137 @@
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="D7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="D8" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="D9" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="D10" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="D12" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="D13" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="D14" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>3</v>

</xml_diff>